<commit_message>
User Stories and Product Backlog updates
</commit_message>
<xml_diff>
--- a/deliverables/Product Backlog-FILLED.xlsx
+++ b/deliverables/Product Backlog-FILLED.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/honesttape/Desktop/ALL/Currents /This Current/Codes/ITSC-3155-Group-Project-Group-19/deliverables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D07081-D277-B541-9DA0-7F0A3A6317DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC300A17-575A-0D46-A53F-E1EBF3106F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="17320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="29">
   <si>
     <t>ITSC-3155 Software Engineering</t>
   </si>
@@ -73,7 +73,7 @@
     <t>Real-time order status tracking by order #</t>
   </si>
   <si>
-    <t>Payment processing (multiple methods)</t>
+    <t>Payment processing (multiple methods, transaction status, failures)</t>
   </si>
   <si>
     <t>Staff views for order management</t>
@@ -85,13 +85,13 @@
     <t>Chef/kitchen view for incoming orders</t>
   </si>
   <si>
-    <t>Customer reviews &amp; ratings</t>
+    <t>Customer reviews &amp; ratings (one review per order)</t>
   </si>
   <si>
     <t>No</t>
   </si>
   <si>
-    <t>Promotions &amp; promo code generation</t>
+    <t>Promotions: create codes; validate &amp; apply at checkout</t>
   </si>
   <si>
     <t>Analytics: trends, preferences, sales</t>
@@ -101,13 +101,19 @@
   </si>
   <si>
     <t>Documentation &amp; staff training materials</t>
+  </si>
+  <si>
+    <t>Order record: customer link, total price, status, tracking #, order type</t>
+  </si>
+  <si>
+    <t>Staff &amp; cook: update order status</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -115,26 +121,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="&quot;⋎ntury Gothic\&quot;&quot;"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="&quot;⋎ntury Gothic\&quot;&quot;"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -229,24 +231,24 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -467,333 +469,375 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="42.1640625" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="18.5" customWidth="1"/>
+    <col min="1" max="1" width="42.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="1"/>
+    <col min="3" max="3" width="14.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="12.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1">
-      <c r="A2" s="4" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:6" ht="13">
-      <c r="A3" s="1" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="13">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="10">
         <v>8</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="3">
+      <c r="D4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="13">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A5" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="10">
         <v>8</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3">
+      <c r="D5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="13">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="10">
         <v>13</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F6" s="3">
+      <c r="D6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="13">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="10">
         <v>8</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="3">
+      <c r="D7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="13">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="10">
         <v>5</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="3">
+      <c r="D8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="13">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="3">
+      <c r="C9" s="10">
         <v>3</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="3">
+      <c r="D9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="13">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A10" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="10">
         <v>8</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="3">
+      <c r="D10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="13">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C11" s="10">
         <v>13</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="3">
+      <c r="D11" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="10">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="13">
-      <c r="A12" s="2" t="s">
+    <row r="12" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="10">
         <v>8</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F12" s="3">
+      <c r="D12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="10">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="13">
-      <c r="A13" s="2" t="s">
+    <row r="13" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="10">
         <v>5</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="3">
+      <c r="D13" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="10">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="13">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A14" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14" s="10">
         <v>8</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="D14" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="10">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="13">
-      <c r="A15" s="2" t="s">
+    <row r="15" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="10">
         <v>8</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="D15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="10">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="13">
-      <c r="A16" s="9" t="s">
+    <row r="16" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B16" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="2">
         <v>13</v>
       </c>
-      <c r="D16" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="9" t="s">
+      <c r="D16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="10">
+      <c r="F16" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="13">
-      <c r="A17" s="9" t="s">
+    <row r="17" spans="1:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="2">
         <v>5</v>
       </c>
-      <c r="D17" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="9" t="s">
+      <c r="D17" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="2">
         <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="13" x14ac:dyDescent="0.15">
+      <c r="A18" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="2">
+        <v>8</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="13" x14ac:dyDescent="0.15">
+      <c r="A19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="2">
+        <v>3</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="2">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>